<commit_message>
fix các biểu mẫu theo ISO
</commit_message>
<xml_diff>
--- a/dataproduct.api/wwwroot/templates/HRC1_BB_NauLuyen_BOF.xlsx
+++ b/dataproduct.api/wwwroot/templates/HRC1_BB_NauLuyen_BOF.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15040D97-6C55-429D-9004-81EBE5AECD3B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2FC9A91-2A4D-4609-806F-5DADE5F9B396}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,9 +22,9 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
   <si>
-    <t>BM.08/QT.05.15
-Ngày hiệu lực: 10/01/2025
-Lần sửa đổi: 00</t>
+    <t>BM.07/QT.05.10
+Ngày hiệu lực: 01/07/2024
+Lần sửa đổi: 02</t>
   </si>
 </sst>
 </file>
@@ -97,15 +97,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>101022</xdr:colOff>
+      <xdr:colOff>274204</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>144319</xdr:rowOff>
+      <xdr:rowOff>216478</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>404091</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>716345</xdr:rowOff>
+      <xdr:colOff>577273</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>23617</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -128,7 +128,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="101022" y="144319"/>
+          <a:off x="274204" y="216478"/>
           <a:ext cx="2424546" cy="1033844"/>
         </a:xfrm>
         <a:prstGeom prst="rect">

</xml_diff>